<commit_message>
progress: 35 village workbooks (randomwalk-TRX50-WS 2026-10-09T15:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
@@ -1142,11 +1142,6 @@
           <t>152</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1154,11 +1149,6 @@
           <t>153</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1166,11 +1156,6 @@
           <t>154</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 4A, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1178,11 +1163,6 @@
           <t>156</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5A, 5B, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1190,11 +1170,6 @@
           <t>157</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1202,11 +1177,6 @@
           <t>158</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1214,11 +1184,6 @@
           <t>159</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1226,11 +1191,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13A, 13B, 1A, 1B, 2, 3A, 3B, 3C, 4A, 4B, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1238,11 +1198,6 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1A1A1, 1A1B, 1A1C, 1A2, 1B, 2, 3A, 3B, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1250,11 +1205,6 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24A1, 24A2, 24A3, 24A4, 24A5, 24A6, 3, 4A, 4B, 5A, 5B, 5C, 6, 7A1, 7A2, 7A3, 7A4, 8, 9A1, 9A2, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1262,11 +1212,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>19B, 1A1, 1A2, 2A, 2B, 3A1, 3A2, 3A3, 3B, 4, 5A, 5B, 5C, 6, 7A, 7B</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1274,11 +1219,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1286,11 +1226,6 @@
           <t>20</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>10, 1A, 1B, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 7A, 7B1, 7B2, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1298,11 +1233,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A1, 3A2, 3A3, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1310,11 +1240,6 @@
           <t>22</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B1A, 3B1B, 3B1C1, 3B1C2, 3B2, 3B3A1A, 3B3A2, 4, 5A, 5B, 5C, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1322,11 +1247,6 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1334,11 +1254,6 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A, 17B, 17B1, 17B2, 17B3, 17B4, 17B5, 17B6, 18B, 19, 20A, 20B1, 20B2, 21A, 21B, 21C, 22, 23, 24, 25A, 25B, 26, 27, 28, 29, 2A, 2B, 2C, 3, 30, 31, 32A, 32B, 33, 34, 35, 36, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1346,11 +1261,6 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17A, 17B, 18, 19A, 19B, 19C, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1358,11 +1268,6 @@
           <t>26</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 2A, 2B, 3, 4A, 4B, 5A, 5B, 5C, 5D, 6A, 6B, 7A, 7B1, 7B2, 7C1, 7C2, 7D1A, 7D1B, 7D2, 8A, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1370,11 +1275,6 @@
           <t>27</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2A1, 2A2, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1382,11 +1282,6 @@
           <t>28</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B, 2C, 2D, 3, 4A, 4B, 5</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1394,11 +1289,6 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 2, 3, 4, 5, 6A1, 6A2A, 6A2B, 6A2C, 6A2D, 6B, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1406,11 +1296,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1418,11 +1303,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1430,11 +1310,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>10, 1A, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1442,11 +1317,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1454,11 +1324,6 @@
           <t>33</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1466,11 +1331,6 @@
           <t>34</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1478,11 +1338,6 @@
           <t>35</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1490,11 +1345,6 @@
           <t>36</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>10, 1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1502,11 +1352,6 @@
           <t>37</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1514,11 +1359,6 @@
           <t>38</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1526,11 +1366,6 @@
           <t>39</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1538,11 +1373,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1550,11 +1380,6 @@
           <t>40</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1562,11 +1387,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1574,11 +1394,6 @@
           <t>42</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 7C</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1586,11 +1401,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B, 1C, 2</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1598,11 +1408,6 @@
           <t>44</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1610,11 +1415,6 @@
           <t>45</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1622,11 +1422,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1634,11 +1429,6 @@
           <t>47</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1646,11 +1436,6 @@
           <t>48</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1658,11 +1443,6 @@
           <t>49</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1670,11 +1450,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1682,11 +1457,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1694,11 +1464,6 @@
           <t>51</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1706,11 +1471,6 @@
           <t>52</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1718,11 +1478,6 @@
           <t>53</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1730,11 +1485,6 @@
           <t>54</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1742,11 +1492,6 @@
           <t>55</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 2A, 2B, 3A, 3B, 4A1, 4A2</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1754,11 +1499,6 @@
           <t>56</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1766,11 +1506,6 @@
           <t>57</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1778,11 +1513,6 @@
           <t>58</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1790,11 +1520,6 @@
           <t>59</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1802,11 +1527,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1814,11 +1534,6 @@
           <t>60</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1826,11 +1541,6 @@
           <t>61</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1838,11 +1548,6 @@
           <t>62</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1850,11 +1555,6 @@
           <t>63</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1862,11 +1562,6 @@
           <t>64</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1874,11 +1569,6 @@
           <t>65</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B, 3</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1886,11 +1576,6 @@
           <t>66</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1898,11 +1583,6 @@
           <t>67</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1910,11 +1590,6 @@
           <t>68</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1922,11 +1597,6 @@
           <t>69</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1934,11 +1604,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4, 5, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1946,11 +1611,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3, 4A, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1958,11 +1618,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1970,11 +1625,6 @@
           <t>72</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1982,11 +1632,6 @@
           <t>73</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A1, 4A2, 4B, 5A, 5B, 5C</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1994,11 +1639,6 @@
           <t>74</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B1, 5B2, 6, 7A, 7B, 7C</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2006,11 +1646,6 @@
           <t>75</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2018,11 +1653,6 @@
           <t>76</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2030,11 +1660,6 @@
           <t>77</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2042,11 +1667,6 @@
           <t>78</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2054,11 +1674,6 @@
           <t>79</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3, 4A, 4B, 5A, 5B, 5C, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2066,11 +1681,6 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A1, 8A2, 8B1, 8B2, 8B3, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2078,11 +1688,6 @@
           <t>80</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 6</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2090,11 +1695,6 @@
           <t>81</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2102,11 +1702,6 @@
           <t>82</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2114,11 +1709,6 @@
           <t>83</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2126,11 +1716,6 @@
           <t>84</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2138,11 +1723,6 @@
           <t>85</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2A, 2B, 2C, 3</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2150,11 +1730,6 @@
           <t>86</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2162,11 +1737,6 @@
           <t>88</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2174,11 +1744,6 @@
           <t>89</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2186,11 +1751,6 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>1, 10A1, 10A2, 10B, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2198,11 +1758,6 @@
           <t>90</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2210,11 +1765,6 @@
           <t>91</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 5D, 6A, 6B, 6C1, 6C2, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2222,11 +1772,6 @@
           <t>92</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2234,11 +1779,6 @@
           <t>93</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2246,11 +1786,6 @@
           <t>94</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2258,11 +1793,6 @@
           <t>95</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2270,11 +1800,6 @@
           <t>96</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2282,11 +1807,6 @@
           <t>97</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2294,21 +1814,11 @@
           <t>98</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
           <t>99</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 36 village workbooks (randomwalk-TRX50-WS 2026-10-09T15:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
@@ -1142,6 +1142,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1149,6 +1154,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1156,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1163,6 +1178,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1170,6 +1190,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1177,6 +1202,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1184,6 +1214,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1191,6 +1226,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 1A, 1B, 2, 3A, 3B, 3C, 4A, 4B, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1198,6 +1238,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1B, 1A1C, 1A2, 1B, 2, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1205,6 +1250,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24A1, 24A2, 24A3, 24A4, 24A5, 24A6, 3, 4A, 4B, 5A, 5B, 5C, 6, 7A1, 7A2, 7A3, 7A4, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1212,6 +1262,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>19B, 1A1, 1A2, 2A, 2B, 3A1, 3A2, 3A3, 3B, 4, 5A, 5B, 5C, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1219,6 +1274,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1226,6 +1286,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 7A, 7B1, 7B2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1233,6 +1298,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A1, 3A2, 3A3, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1240,6 +1310,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1A, 3B1B, 3B1C1, 3B1C2, 3B2, 3B3A1A, 3B3A2, 4, 5A, 5B, 5C, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1247,6 +1322,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1254,6 +1334,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A, 17B, 17B1, 17B2, 17B3, 17B4, 17B5, 17B6, 18B, 19, 20A, 20B1, 20B2, 21A, 21B, 21C, 22, 23, 24, 25A, 25B, 26, 27, 28, 29, 2A, 2B, 2C, 3, 30, 31, 32A, 32B, 33, 34, 35, 36, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1261,6 +1346,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17A, 17B, 18, 19A, 19B, 19C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1268,6 +1358,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 2A, 2B, 3, 4A, 4B, 5A, 5B, 5C, 5D, 6A, 6B, 7A, 7B1, 7B2, 7C1, 7C2, 7D1A, 7D1B, 7D2, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1275,6 +1370,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1282,6 +1382,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1289,6 +1394,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 2, 3, 4, 5, 6A1, 6A2A, 6A2B, 6A2C, 6A2D, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1296,6 +1406,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1303,6 +1418,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1310,6 +1430,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1317,6 +1442,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1324,6 +1454,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1331,6 +1466,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1338,6 +1478,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1345,6 +1490,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1352,6 +1502,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1359,6 +1514,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1366,6 +1526,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1373,6 +1538,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1380,6 +1550,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1387,6 +1562,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1394,6 +1574,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1401,6 +1586,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1408,6 +1598,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1415,6 +1610,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1422,6 +1622,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1429,6 +1634,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1436,6 +1646,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1443,6 +1658,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1450,6 +1670,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1457,6 +1682,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1464,6 +1694,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1471,6 +1706,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1478,6 +1718,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1485,6 +1730,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1492,6 +1742,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 2A, 2B, 3A, 3B, 4A1, 4A2</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1499,6 +1754,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1506,6 +1766,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1513,6 +1778,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1520,6 +1790,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1527,6 +1802,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1534,6 +1814,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1541,6 +1826,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1548,6 +1838,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1555,6 +1850,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1562,6 +1862,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1569,6 +1874,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1576,6 +1886,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1583,6 +1898,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1590,6 +1910,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1597,6 +1922,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1604,6 +1934,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1611,6 +1946,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1618,6 +1958,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1625,6 +1970,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1632,6 +1982,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A1, 4A2, 4B, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1639,6 +1994,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B1, 5B2, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1646,6 +2006,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1653,6 +2018,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1660,6 +2030,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1667,6 +2042,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1674,6 +2054,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4A, 4B, 5A, 5B, 5C, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1681,6 +2066,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A1, 8A2, 8B1, 8B2, 8B3, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1688,6 +2078,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1695,6 +2090,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1702,6 +2102,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1709,6 +2114,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1716,6 +2126,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1723,6 +2138,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1730,6 +2150,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1737,6 +2162,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1744,6 +2174,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1751,6 +2186,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10B, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1758,6 +2198,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1765,6 +2210,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 5D, 6A, 6B, 6C1, 6C2, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1772,6 +2222,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1779,6 +2234,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -1786,6 +2246,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -1793,6 +2258,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -1800,6 +2270,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -1807,11 +2282,21 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
           <t>98</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3, 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 38 village workbooks (randomwalk-TRX50-WS 2026-10-09T16:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
@@ -2306,6 +2306,11 @@
           <t>99</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
progress: 33 village workbooks (rw-rtx-3070 2026-10-09T21:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
@@ -746,6 +746,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -753,6 +758,11 @@
           <t>123</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -760,6 +770,11 @@
           <t>124</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -767,6 +782,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -774,6 +794,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -781,6 +806,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -788,6 +818,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -795,6 +830,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10, 11, 12A1, 12A2, 12A3, 12B, 12C1, 12C2, 12C3, 12C4, 13A1, 13D, 14A1, 14A2, 14A3, 14A4, 1A, 1B, 2A, 2B, 3A, 3B1, 3B2, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -802,6 +842,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B1, 1B2, 2A, 2B1, 2B2, 3, 4A1, 4A2, 4A3, 4B1, 4B2, 4B3, 4C, 5, 6A1, 6A2, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -809,6 +854,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B, 2C, 2D1, 2D2, 2E, 2F</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -816,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -823,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -830,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -837,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -844,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -851,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 6A1, 6B, 6C</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -858,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -865,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -872,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -879,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 10D, 11A1, 11A2, 11B, 12, 13, 14, 15, 1A, 1B, 1C, 2A, 2B, 2C, 3, 4A, 4B, 5, 6A1, 6A2, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -886,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -893,6 +998,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -900,6 +1010,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -907,6 +1022,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -914,6 +1034,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -921,6 +1046,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -928,6 +1058,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B1, 3B2, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -935,6 +1070,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -942,6 +1082,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -949,6 +1094,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -956,6 +1106,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -963,6 +1118,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -970,6 +1130,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -977,6 +1142,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -984,6 +1154,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -991,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -998,6 +1178,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1005,6 +1190,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1012,6 +1202,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1019,6 +1214,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1026,6 +1226,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 1A, 1B, 2, 3A, 3B, 3C, 4A, 4B, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1033,6 +1238,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1B, 1A1C, 1A2, 1B, 2, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1040,6 +1250,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24A1, 24A2, 24A3, 24A4, 24A5, 24A6, 3, 4A, 4B, 5A, 5B, 5C, 6, 7A1, 7A2, 7A3, 7A4, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1047,6 +1262,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>19B, 1A1, 1A2, 2A, 2B, 3A1, 3A2, 3A3, 3B, 4, 5A, 5B, 5C, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1054,6 +1274,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1061,6 +1286,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 7A, 7B1, 7B2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1068,6 +1298,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A1, 3A2, 3A3, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1075,6 +1310,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1A, 3B1B, 3B1C1, 3B1C2, 3B2, 3B3A1A, 3B3A2, 4, 5A, 5B, 5C, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1082,6 +1322,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1089,6 +1334,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A, 17B, 17B1, 17B2, 17B3, 17B4, 17B5, 17B6, 18B, 19, 20A, 20B1, 20B2, 21A, 21B, 21C, 22, 23, 24, 25A, 25B, 26, 27, 28, 29, 2A, 2B, 2C, 3, 30, 31, 32A, 32B, 33, 34, 35, 36, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1096,6 +1346,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17A, 17B, 18, 19A, 19B, 19C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1103,6 +1358,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 2A, 2B, 3, 4A, 4B, 5A, 5B, 5C, 5D, 6A, 6B, 7A, 7B1, 7B2, 7C1, 7C2, 7D1A, 7D1B, 7D2, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1110,6 +1370,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1117,6 +1382,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1124,6 +1394,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 2, 3, 4, 5, 6A1, 6A2A, 6A2B, 6A2C, 6A2D, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1131,6 +1406,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1138,6 +1418,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1145,6 +1430,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1152,6 +1442,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1159,6 +1454,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1166,6 +1466,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1173,6 +1478,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1180,6 +1490,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1187,6 +1502,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1194,6 +1514,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1201,6 +1526,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1208,6 +1538,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1215,6 +1550,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1222,6 +1562,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1229,6 +1574,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1236,6 +1586,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1243,6 +1598,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1250,6 +1610,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1257,6 +1622,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1264,6 +1634,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1271,6 +1646,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1278,6 +1658,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1285,6 +1670,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1292,6 +1682,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1299,6 +1694,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1306,6 +1706,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1313,6 +1718,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1320,6 +1730,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1327,6 +1742,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 2A, 2B, 3A, 3B, 4A1, 4A2</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1334,6 +1754,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1341,6 +1766,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1348,6 +1778,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1355,6 +1790,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1362,6 +1802,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1369,6 +1814,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1376,6 +1826,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1383,11 +1838,21 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
           <t>63</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 34 village workbooks (rw-rtx-3070 2026-10-09T22:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Appavaram_13.454424_80.159516.xlsx
@@ -1862,6 +1862,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1869,6 +1874,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1876,6 +1886,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1883,6 +1898,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1890,6 +1910,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1897,6 +1922,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1904,6 +1934,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1911,6 +1946,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1918,6 +1958,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1925,6 +1970,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1932,6 +1982,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A1, 4A2, 4B, 5A, 5B, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1939,6 +1994,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B1, 5B2, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1946,6 +2006,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1953,6 +2018,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1960,6 +2030,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1967,6 +2042,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1974,6 +2054,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4A, 4B, 5A, 5B, 5C, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1981,6 +2066,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A1, 8A2, 8B1, 8B2, 8B3, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1988,6 +2078,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1995,6 +2090,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2002,6 +2102,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2009,6 +2114,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2016,6 +2126,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2023,6 +2138,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2030,6 +2150,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2037,6 +2162,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2044,6 +2174,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2051,6 +2186,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10B, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2058,6 +2198,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2065,6 +2210,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 5D, 6A, 6B, 6C1, 6C2, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2072,6 +2222,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2079,6 +2234,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2086,6 +2246,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2093,6 +2258,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2100,6 +2270,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2107,6 +2282,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2114,11 +2294,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>